<commit_message>
teste de nsga falhou
</commit_message>
<xml_diff>
--- a/tests/correcoes_resultantes.xlsx
+++ b/tests/correcoes_resultantes.xlsx
@@ -490,25 +490,25 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>29</v>
+        <v>30.25</v>
       </c>
       <c r="E2" t="n">
-        <v>9</v>
+        <v>10.25</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0124648341594097</v>
+        <v>0.008964630206430135</v>
       </c>
       <c r="G2" t="n">
-        <v>0.07338950349587595</v>
+        <v>0.07549328792992646</v>
       </c>
       <c r="H2" t="n">
-        <v>0.03510827853583724</v>
+        <v>0.02980551051688964</v>
       </c>
       <c r="I2" t="n">
-        <v>0.8584821428571429</v>
+        <v>0.9488095238095238</v>
       </c>
       <c r="J2" t="n">
-        <v>0.1415178571428571</v>
+        <v>0.05119047619047619</v>
       </c>
     </row>
     <row r="3">
@@ -526,25 +526,25 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>18.09696107085386</v>
+        <v>16.34587103827753</v>
       </c>
       <c r="E3" t="n">
-        <v>6.96419413859206</v>
+        <v>7.154544010627093</v>
       </c>
       <c r="F3" t="n">
-        <v>0.01036887451212508</v>
+        <v>0.006886519703788971</v>
       </c>
       <c r="G3" t="n">
-        <v>0.01633030044745003</v>
+        <v>0.01487575421185004</v>
       </c>
       <c r="H3" t="n">
-        <v>0.02597428100643959</v>
+        <v>0.00652378263345612</v>
       </c>
       <c r="I3" t="n">
-        <v>0.1228992803050115</v>
+        <v>0.05567306167185675</v>
       </c>
       <c r="J3" t="n">
-        <v>0.1228992803050115</v>
+        <v>0.05567306167185677</v>
       </c>
     </row>
     <row r="4">
@@ -562,25 +562,25 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>327.5</v>
+        <v>267.1875</v>
       </c>
       <c r="E4" t="n">
-        <v>48.5</v>
+        <v>51.1875</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0001075135586481972</v>
+        <v>4.742415363067375e-05</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0002666787127039868</v>
+        <v>0.0002212880633713741</v>
       </c>
       <c r="H4" t="n">
-        <v>0.0006746632738014887</v>
+        <v>4.255973984858367e-05</v>
       </c>
       <c r="I4" t="n">
-        <v>0.01510423309948979</v>
+        <v>0.003099489795918365</v>
       </c>
       <c r="J4" t="n">
-        <v>0.0151042330994898</v>
+        <v>0.003099489795918367</v>
       </c>
     </row>
     <row r="5">
@@ -598,25 +598,25 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>18.75</v>
+        <v>17.25</v>
       </c>
       <c r="E5" t="n">
-        <v>4.75</v>
+        <v>5.25</v>
       </c>
       <c r="F5" t="n">
-        <v>0.008970544484396506</v>
+        <v>0.003783025051187017</v>
       </c>
       <c r="G5" t="n">
-        <v>0.08847281204789581</v>
+        <v>0.09056627207516471</v>
       </c>
       <c r="H5" t="n">
-        <v>0.01633116776261659</v>
+        <v>0.01817502945571112</v>
       </c>
       <c r="I5" t="n">
-        <v>0.6186011904761904</v>
+        <v>0.596875</v>
       </c>
       <c r="J5" t="n">
-        <v>0.3813988095238095</v>
+        <v>0.403125</v>
       </c>
     </row>
     <row r="6">
@@ -634,25 +634,25 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>12.77448629104122</v>
+        <v>11.12148820976761</v>
       </c>
       <c r="E6" t="n">
-        <v>4.493050188902857</v>
+        <v>4.968651728587948</v>
       </c>
       <c r="F6" t="n">
-        <v>0.002954046003041886</v>
+        <v>0.002452627372149072</v>
       </c>
       <c r="G6" t="n">
-        <v>0.005554658981901795</v>
+        <v>0.007380678717552542</v>
       </c>
       <c r="H6" t="n">
-        <v>0.01498224500684445</v>
+        <v>0.01723250686056433</v>
       </c>
       <c r="I6" t="n">
-        <v>0.2695690582153464</v>
+        <v>0.2640393850829834</v>
       </c>
       <c r="J6" t="n">
-        <v>0.2695690582153464</v>
+        <v>0.2640393850829834</v>
       </c>
     </row>
     <row r="7">
@@ -670,25 +670,25 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>163.1875</v>
+        <v>123.6875</v>
       </c>
       <c r="E7" t="n">
-        <v>20.1875</v>
+        <v>24.6875</v>
       </c>
       <c r="F7" t="n">
-        <v>8.726387788087743e-06</v>
+        <v>6.015381026614861e-06</v>
       </c>
       <c r="G7" t="n">
-        <v>3.085423640522228e-05</v>
+        <v>5.447441833173302e-05</v>
       </c>
       <c r="H7" t="n">
-        <v>0.0002244676654451156</v>
+        <v>0.0002969592926993967</v>
       </c>
       <c r="I7" t="n">
-        <v>0.07266747714710885</v>
+        <v>0.069716796875</v>
       </c>
       <c r="J7" t="n">
-        <v>0.07266747714710883</v>
+        <v>0.06971679687499999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
atualização do código nsga II
</commit_message>
<xml_diff>
--- a/tests/correcoes_resultantes.xlsx
+++ b/tests/correcoes_resultantes.xlsx
@@ -490,25 +490,25 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>30.25</v>
+        <v>29.5</v>
       </c>
       <c r="E2" t="n">
-        <v>10.25</v>
+        <v>9.25</v>
       </c>
       <c r="F2" t="n">
-        <v>0.008964630206430135</v>
+        <v>0.007904201470481757</v>
       </c>
       <c r="G2" t="n">
-        <v>0.07549328792992646</v>
+        <v>0.07267255956850993</v>
       </c>
       <c r="H2" t="n">
-        <v>0.02980551051688964</v>
+        <v>0.02636513592118675</v>
       </c>
       <c r="I2" t="n">
-        <v>0.9488095238095238</v>
+        <v>0.9133928571428571</v>
       </c>
       <c r="J2" t="n">
-        <v>0.05119047619047619</v>
+        <v>0.08660714285714285</v>
       </c>
     </row>
     <row r="3">
@@ -526,25 +526,25 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>16.34587103827753</v>
+        <v>16.68082731761228</v>
       </c>
       <c r="E3" t="n">
-        <v>7.154544010627093</v>
+        <v>8.011710179481033</v>
       </c>
       <c r="F3" t="n">
-        <v>0.006886519703788971</v>
+        <v>0.007068114810640908</v>
       </c>
       <c r="G3" t="n">
-        <v>0.01487575421185004</v>
+        <v>0.02276598273197072</v>
       </c>
       <c r="H3" t="n">
-        <v>0.00652378263345612</v>
+        <v>0.01083019523964862</v>
       </c>
       <c r="I3" t="n">
-        <v>0.05567306167185675</v>
+        <v>0.09775460608178052</v>
       </c>
       <c r="J3" t="n">
-        <v>0.05567306167185677</v>
+        <v>0.09775460608178052</v>
       </c>
     </row>
     <row r="4">
@@ -562,25 +562,25 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>267.1875</v>
+        <v>278.25</v>
       </c>
       <c r="E4" t="n">
-        <v>51.1875</v>
+        <v>64.1875</v>
       </c>
       <c r="F4" t="n">
-        <v>4.742415363067375e-05</v>
+        <v>4.995824697640136e-05</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0002212880633713741</v>
+        <v>0.000518289969752389</v>
       </c>
       <c r="H4" t="n">
-        <v>4.255973984858367e-05</v>
+        <v>0.0001172931289289076</v>
       </c>
       <c r="I4" t="n">
-        <v>0.003099489795918365</v>
+        <v>0.009555963010204081</v>
       </c>
       <c r="J4" t="n">
-        <v>0.003099489795918367</v>
+        <v>0.009555963010204081</v>
       </c>
     </row>
     <row r="5">
@@ -598,25 +598,25 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>17.25</v>
+        <v>17.5</v>
       </c>
       <c r="E5" t="n">
-        <v>5.25</v>
+        <v>5</v>
       </c>
       <c r="F5" t="n">
-        <v>0.003783025051187017</v>
+        <v>0.008275664561183711</v>
       </c>
       <c r="G5" t="n">
-        <v>0.09056627207516471</v>
+        <v>0.08607363256516801</v>
       </c>
       <c r="H5" t="n">
-        <v>0.01817502945571112</v>
+        <v>0.01677053507368865</v>
       </c>
       <c r="I5" t="n">
-        <v>0.596875</v>
+        <v>0.5894345238095238</v>
       </c>
       <c r="J5" t="n">
-        <v>0.403125</v>
+        <v>0.4105654761904762</v>
       </c>
     </row>
     <row r="6">
@@ -634,25 +634,25 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>11.12148820976761</v>
+        <v>10.98863048791796</v>
       </c>
       <c r="E6" t="n">
-        <v>4.968651728587948</v>
+        <v>4.847679857416329</v>
       </c>
       <c r="F6" t="n">
-        <v>0.002452627372149072</v>
+        <v>0.005507855474296813</v>
       </c>
       <c r="G6" t="n">
-        <v>0.007380678717552542</v>
+        <v>0.0119021731342456</v>
       </c>
       <c r="H6" t="n">
-        <v>0.01723250686056433</v>
+        <v>0.0150891972486803</v>
       </c>
       <c r="I6" t="n">
-        <v>0.2640393850829834</v>
+        <v>0.2814319375629606</v>
       </c>
       <c r="J6" t="n">
-        <v>0.2640393850829834</v>
+        <v>0.2814319375629606</v>
       </c>
     </row>
     <row r="7">
@@ -670,25 +670,25 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>123.6875</v>
+        <v>120.75</v>
       </c>
       <c r="E7" t="n">
-        <v>24.6875</v>
+        <v>23.5</v>
       </c>
       <c r="F7" t="n">
-        <v>6.015381026614861e-06</v>
+        <v>3.033647192574137e-05</v>
       </c>
       <c r="G7" t="n">
-        <v>5.447441833173302e-05</v>
+        <v>0.0001416617253175578</v>
       </c>
       <c r="H7" t="n">
-        <v>0.0002969592926993967</v>
+        <v>0.0002276838736095813</v>
       </c>
       <c r="I7" t="n">
-        <v>0.069716796875</v>
+        <v>0.07920393548044219</v>
       </c>
       <c r="J7" t="n">
-        <v>0.06971679687499999</v>
+        <v>0.07920393548044216</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
test nsga result V and VI
</commit_message>
<xml_diff>
--- a/tests/correcoes_resultantes.xlsx
+++ b/tests/correcoes_resultantes.xlsx
@@ -490,25 +490,25 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>29.5</v>
+        <v>29.75</v>
       </c>
       <c r="E2" t="n">
-        <v>9.25</v>
+        <v>10</v>
       </c>
       <c r="F2" t="n">
-        <v>0.007904201470481757</v>
+        <v>0.007124433247613776</v>
       </c>
       <c r="G2" t="n">
-        <v>0.07267255956850993</v>
+        <v>0.08487814078301652</v>
       </c>
       <c r="H2" t="n">
-        <v>0.02636513592118675</v>
+        <v>0.03224753527760904</v>
       </c>
       <c r="I2" t="n">
-        <v>0.9133928571428571</v>
+        <v>0.9485119047619048</v>
       </c>
       <c r="J2" t="n">
-        <v>0.08660714285714285</v>
+        <v>0.05148809523809524</v>
       </c>
     </row>
     <row r="3">
@@ -526,25 +526,25 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>16.68082731761228</v>
+        <v>15.46568782822154</v>
       </c>
       <c r="E3" t="n">
-        <v>8.011710179481033</v>
+        <v>6.403124237432849</v>
       </c>
       <c r="F3" t="n">
-        <v>0.007068114810640908</v>
+        <v>0.001154883754579223</v>
       </c>
       <c r="G3" t="n">
-        <v>0.02276598273197072</v>
+        <v>0.009077775791329521</v>
       </c>
       <c r="H3" t="n">
-        <v>0.01083019523964862</v>
+        <v>0.0108344010726961</v>
       </c>
       <c r="I3" t="n">
-        <v>0.09775460608178052</v>
+        <v>0.0328340045340421</v>
       </c>
       <c r="J3" t="n">
-        <v>0.09775460608178052</v>
+        <v>0.0328340045340421</v>
       </c>
     </row>
     <row r="4">
@@ -562,25 +562,25 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>278.25</v>
+        <v>239.1875</v>
       </c>
       <c r="E4" t="n">
-        <v>64.1875</v>
+        <v>41</v>
       </c>
       <c r="F4" t="n">
-        <v>4.995824697640136e-05</v>
+        <v>1.333756486591003e-06</v>
       </c>
       <c r="G4" t="n">
-        <v>0.000518289969752389</v>
+        <v>8.24060133176483e-05</v>
       </c>
       <c r="H4" t="n">
-        <v>0.0001172931289289076</v>
+        <v>0.0001173842466040383</v>
       </c>
       <c r="I4" t="n">
-        <v>0.009555963010204081</v>
+        <v>0.001078071853741497</v>
       </c>
       <c r="J4" t="n">
-        <v>0.009555963010204081</v>
+        <v>0.001078071853741497</v>
       </c>
     </row>
     <row r="5">
@@ -598,25 +598,25 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>17.5</v>
+        <v>18.25</v>
       </c>
       <c r="E5" t="n">
-        <v>5</v>
+        <v>6.75</v>
       </c>
       <c r="F5" t="n">
-        <v>0.008275664561183711</v>
+        <v>0.009063596605706265</v>
       </c>
       <c r="G5" t="n">
-        <v>0.08607363256516801</v>
+        <v>0.08528570052064546</v>
       </c>
       <c r="H5" t="n">
-        <v>0.01677053507368865</v>
+        <v>0.02081123332214346</v>
       </c>
       <c r="I5" t="n">
-        <v>0.5894345238095238</v>
+        <v>0.6334821428571429</v>
       </c>
       <c r="J5" t="n">
-        <v>0.4105654761904762</v>
+        <v>0.3665178571428572</v>
       </c>
     </row>
     <row r="6">
@@ -634,25 +634,25 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>10.98863048791796</v>
+        <v>9.653367288153911</v>
       </c>
       <c r="E6" t="n">
-        <v>4.847679857416329</v>
+        <v>7.189401922274203</v>
       </c>
       <c r="F6" t="n">
-        <v>0.005507855474296813</v>
+        <v>0.005327922554336107</v>
       </c>
       <c r="G6" t="n">
-        <v>0.0119021731342456</v>
+        <v>0.009175202168653336</v>
       </c>
       <c r="H6" t="n">
-        <v>0.0150891972486803</v>
+        <v>0.01825308117920165</v>
       </c>
       <c r="I6" t="n">
-        <v>0.2814319375629606</v>
+        <v>0.210371145392555</v>
       </c>
       <c r="J6" t="n">
-        <v>0.2814319375629606</v>
+        <v>0.210371145392555</v>
       </c>
     </row>
     <row r="7">
@@ -670,25 +670,25 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>120.75</v>
+        <v>93.1875</v>
       </c>
       <c r="E7" t="n">
-        <v>23.5</v>
+        <v>51.6875</v>
       </c>
       <c r="F7" t="n">
-        <v>3.033647192574137e-05</v>
+        <v>2.838675874500339e-05</v>
       </c>
       <c r="G7" t="n">
-        <v>0.0001416617253175578</v>
+        <v>8.418433483566089e-05</v>
       </c>
       <c r="H7" t="n">
-        <v>0.0002276838736095813</v>
+        <v>0.0003331749725345255</v>
       </c>
       <c r="I7" t="n">
-        <v>0.07920393548044219</v>
+        <v>0.04425601881377551</v>
       </c>
       <c r="J7" t="n">
-        <v>0.07920393548044216</v>
+        <v>0.04425601881377551</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
resultado final com resultado nsga VII
</commit_message>
<xml_diff>
--- a/tests/correcoes_resultantes.xlsx
+++ b/tests/correcoes_resultantes.xlsx
@@ -490,25 +490,25 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>29.75</v>
+        <v>31</v>
       </c>
       <c r="E2" t="n">
-        <v>10</v>
+        <v>8.25</v>
       </c>
       <c r="F2" t="n">
-        <v>0.007124433247613776</v>
+        <v>0.008091809862252393</v>
       </c>
       <c r="G2" t="n">
-        <v>0.08487814078301652</v>
+        <v>0.08874971886813687</v>
       </c>
       <c r="H2" t="n">
-        <v>0.03224753527760904</v>
+        <v>0.02434549439225434</v>
       </c>
       <c r="I2" t="n">
-        <v>0.9485119047619048</v>
+        <v>0.9754464285714286</v>
       </c>
       <c r="J2" t="n">
-        <v>0.05148809523809524</v>
+        <v>0.02455357142857143</v>
       </c>
     </row>
     <row r="3">
@@ -526,25 +526,25 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>15.46568782822154</v>
+        <v>16.74813422444423</v>
       </c>
       <c r="E3" t="n">
-        <v>6.403124237432849</v>
+        <v>6.259992012774457</v>
       </c>
       <c r="F3" t="n">
-        <v>0.001154883754579223</v>
+        <v>0.00380178574539941</v>
       </c>
       <c r="G3" t="n">
-        <v>0.009077775791329521</v>
+        <v>0.006823502354496241</v>
       </c>
       <c r="H3" t="n">
-        <v>0.0108344010726961</v>
+        <v>0.00672443506400267</v>
       </c>
       <c r="I3" t="n">
-        <v>0.0328340045340421</v>
+        <v>0.02631657616640981</v>
       </c>
       <c r="J3" t="n">
-        <v>0.0328340045340421</v>
+        <v>0.02631657616640981</v>
       </c>
     </row>
     <row r="4">
@@ -562,25 +562,25 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>239.1875</v>
+        <v>280.5</v>
       </c>
       <c r="E4" t="n">
-        <v>41</v>
+        <v>39.1875</v>
       </c>
       <c r="F4" t="n">
-        <v>1.333756486591003e-06</v>
+        <v>1.445357485392214e-05</v>
       </c>
       <c r="G4" t="n">
-        <v>8.24060133176483e-05</v>
+        <v>4.656018438181574e-05</v>
       </c>
       <c r="H4" t="n">
-        <v>0.0001173842466040383</v>
+        <v>4.52180269299886e-05</v>
       </c>
       <c r="I4" t="n">
-        <v>0.001078071853741497</v>
+        <v>0.0006925621811224489</v>
       </c>
       <c r="J4" t="n">
-        <v>0.001078071853741497</v>
+        <v>0.0006925621811224489</v>
       </c>
     </row>
     <row r="5">
@@ -598,25 +598,25 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>18.25</v>
+        <v>19</v>
       </c>
       <c r="E5" t="n">
-        <v>6.75</v>
+        <v>4.5</v>
       </c>
       <c r="F5" t="n">
-        <v>0.009063596605706265</v>
+        <v>0.00493200682106875</v>
       </c>
       <c r="G5" t="n">
-        <v>0.08528570052064546</v>
+        <v>0.08941729030528298</v>
       </c>
       <c r="H5" t="n">
-        <v>0.02081123332214346</v>
+        <v>0.01492667338059412</v>
       </c>
       <c r="I5" t="n">
-        <v>0.6334821428571429</v>
+        <v>0.6654761904761906</v>
       </c>
       <c r="J5" t="n">
-        <v>0.3665178571428572</v>
+        <v>0.3345238095238095</v>
       </c>
     </row>
     <row r="6">
@@ -634,25 +634,25 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>9.653367288153911</v>
+        <v>10.88577052853862</v>
       </c>
       <c r="E6" t="n">
-        <v>7.189401922274203</v>
+        <v>4.387482193696061</v>
       </c>
       <c r="F6" t="n">
-        <v>0.005327922554336107</v>
+        <v>0.005224679337844496</v>
       </c>
       <c r="G6" t="n">
-        <v>0.009175202168653336</v>
+        <v>0.01262831277600179</v>
       </c>
       <c r="H6" t="n">
-        <v>0.01825308117920165</v>
+        <v>0.01287609006375795</v>
       </c>
       <c r="I6" t="n">
-        <v>0.210371145392555</v>
+        <v>0.2726983145314605</v>
       </c>
       <c r="J6" t="n">
-        <v>0.210371145392555</v>
+        <v>0.2726983145314604</v>
       </c>
     </row>
     <row r="7">
@@ -670,25 +670,25 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>93.1875</v>
+        <v>118.5</v>
       </c>
       <c r="E7" t="n">
-        <v>51.6875</v>
+        <v>19.25</v>
       </c>
       <c r="F7" t="n">
-        <v>2.838675874500339e-05</v>
+        <v>2.72972741832992e-05</v>
       </c>
       <c r="G7" t="n">
-        <v>8.418433483566089e-05</v>
+        <v>0.0001594742835685302</v>
       </c>
       <c r="H7" t="n">
-        <v>0.0003331749725345255</v>
+        <v>0.0001657936953300063</v>
       </c>
       <c r="I7" t="n">
-        <v>0.04425601881377551</v>
+        <v>0.07436437074829934</v>
       </c>
       <c r="J7" t="n">
-        <v>0.04425601881377551</v>
+        <v>0.07436437074829931</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
tentando gerar a curva de pareto
</commit_message>
<xml_diff>
--- a/tests/correcoes_resultantes.xlsx
+++ b/tests/correcoes_resultantes.xlsx
@@ -490,25 +490,25 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E2" t="n">
-        <v>8.25</v>
+        <v>13.25</v>
       </c>
       <c r="F2" t="n">
-        <v>0.008091809862252393</v>
+        <v>0.02457086813714842</v>
       </c>
       <c r="G2" t="n">
-        <v>0.08874971886813687</v>
+        <v>0.07899207669231606</v>
       </c>
       <c r="H2" t="n">
-        <v>0.02434549439225434</v>
+        <v>0.05008167194259365</v>
       </c>
       <c r="I2" t="n">
-        <v>0.9754464285714286</v>
+        <v>0.9296130952380952</v>
       </c>
       <c r="J2" t="n">
-        <v>0.02455357142857143</v>
+        <v>0.07038690476190476</v>
       </c>
     </row>
     <row r="3">
@@ -526,25 +526,25 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>16.74813422444423</v>
+        <v>16.98528775146303</v>
       </c>
       <c r="E3" t="n">
-        <v>6.259992012774457</v>
+        <v>5.214163403653552</v>
       </c>
       <c r="F3" t="n">
-        <v>0.00380178574539941</v>
+        <v>0.02901793273447585</v>
       </c>
       <c r="G3" t="n">
-        <v>0.006823502354496241</v>
+        <v>0.0164523224561021</v>
       </c>
       <c r="H3" t="n">
-        <v>0.00672443506400267</v>
+        <v>0.0327283586495034</v>
       </c>
       <c r="I3" t="n">
-        <v>0.02631657616640981</v>
+        <v>0.037557530982526</v>
       </c>
       <c r="J3" t="n">
-        <v>0.02631657616640981</v>
+        <v>0.03755753098252601</v>
       </c>
     </row>
     <row r="4">
@@ -562,25 +562,25 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>280.5</v>
+        <v>288.5</v>
       </c>
       <c r="E4" t="n">
-        <v>39.1875</v>
+        <v>27.1875</v>
       </c>
       <c r="F4" t="n">
-        <v>1.445357485392214e-05</v>
+        <v>0.0008420404201825649</v>
       </c>
       <c r="G4" t="n">
-        <v>4.656018438181574e-05</v>
+        <v>0.0002706789141995613</v>
       </c>
       <c r="H4" t="n">
-        <v>4.52180269299886e-05</v>
+        <v>0.001071145459890524</v>
       </c>
       <c r="I4" t="n">
-        <v>0.0006925621811224489</v>
+        <v>0.0014105681335034</v>
       </c>
       <c r="J4" t="n">
-        <v>0.0006925621811224489</v>
+        <v>0.001410568133503401</v>
       </c>
     </row>
     <row r="5">
@@ -598,25 +598,25 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>19</v>
+        <v>16.75</v>
       </c>
       <c r="E5" t="n">
-        <v>4.5</v>
+        <v>6</v>
       </c>
       <c r="F5" t="n">
-        <v>0.00493200682106875</v>
+        <v>0.009243041175822328</v>
       </c>
       <c r="G5" t="n">
-        <v>0.08941729030528298</v>
+        <v>0.0851062559505294</v>
       </c>
       <c r="H5" t="n">
-        <v>0.01492667338059412</v>
+        <v>0.02142338553082812</v>
       </c>
       <c r="I5" t="n">
-        <v>0.6654761904761906</v>
+        <v>0.5703869047619048</v>
       </c>
       <c r="J5" t="n">
-        <v>0.3345238095238095</v>
+        <v>0.4296130952380952</v>
       </c>
     </row>
     <row r="6">
@@ -634,25 +634,25 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>10.88577052853862</v>
+        <v>9.908960591303208</v>
       </c>
       <c r="E6" t="n">
-        <v>4.387482193696061</v>
+        <v>5.612486080160912</v>
       </c>
       <c r="F6" t="n">
-        <v>0.005224679337844496</v>
+        <v>0.005784172408348982</v>
       </c>
       <c r="G6" t="n">
-        <v>0.01262831277600179</v>
+        <v>0.00940770767255405</v>
       </c>
       <c r="H6" t="n">
-        <v>0.01287609006375795</v>
+        <v>0.02171840113295275</v>
       </c>
       <c r="I6" t="n">
-        <v>0.2726983145314605</v>
+        <v>0.2179889884509865</v>
       </c>
       <c r="J6" t="n">
-        <v>0.2726983145314604</v>
+        <v>0.2179889884509866</v>
       </c>
     </row>
     <row r="7">
@@ -670,25 +670,25 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>118.5</v>
+        <v>98.1875</v>
       </c>
       <c r="E7" t="n">
-        <v>19.25</v>
+        <v>31.5</v>
       </c>
       <c r="F7" t="n">
-        <v>2.72972741832992e-05</v>
+        <v>3.345665044950566e-05</v>
       </c>
       <c r="G7" t="n">
-        <v>0.0001594742835685302</v>
+        <v>8.850496365223234e-05</v>
       </c>
       <c r="H7" t="n">
-        <v>0.0001657936953300063</v>
+        <v>0.0004716889477718434</v>
       </c>
       <c r="I7" t="n">
-        <v>0.07436437074829934</v>
+        <v>0.04751919908588435</v>
       </c>
       <c r="J7" t="n">
-        <v>0.07436437074829931</v>
+        <v>0.04751919908588435</v>
       </c>
     </row>
   </sheetData>

</xml_diff>